<commit_message>
funcion de doble tabla
</commit_message>
<xml_diff>
--- a/data/pedidos_2026-08-10.xlsx
+++ b/data/pedidos_2026-08-10.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pedidos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Pedidos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -560,7 +560,7 @@
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>success</t>
         </is>
       </c>
       <c r="P2" t="inlineStr"/>
@@ -627,7 +627,7 @@
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>success</t>
         </is>
       </c>
       <c r="P3" t="inlineStr"/>
@@ -697,7 +697,7 @@
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>success</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -767,7 +767,7 @@
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>success</t>
         </is>
       </c>
       <c r="P5" t="inlineStr"/>
@@ -837,7 +837,7 @@
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>success</t>
         </is>
       </c>
       <c r="P6" t="inlineStr"/>
@@ -907,7 +907,7 @@
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>success</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -977,7 +977,7 @@
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>success</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>

</xml_diff>